<commit_message>
maj de l'estimation avec calcul temps homme
</commit_message>
<xml_diff>
--- a/docs/cadrage/Estimation_NutriScope.xlsx
+++ b/docs/cadrage/Estimation_NutriScope.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t xml:space="preserve">Mois</t>
   </si>
@@ -112,6 +112,30 @@
   <si>
     <t xml:space="preserve">Modele de revenu choisis Freemium : Abonnement a 5euros par mois</t>
   </si>
+  <si>
+    <t xml:space="preserve">Calcul Temps/Homme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 développeurs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Temps : 256h ( 32 jours de TP fois 8h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Majoration : 30 % (temps passé a travaillé sur le projet chez nous)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">((256 * 0,30) + 256) * 3 = 998,4h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arrondis a 1000h </t>
+  </si>
+  <si>
+    <t xml:space="preserve">taux horaire moyen choisis : 50€/h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1000 x 50 = 50000 €</t>
+  </si>
 </sst>
 </file>
 
@@ -124,7 +148,7 @@
     <numFmt numFmtId="167" formatCode="0.00"/>
     <numFmt numFmtId="168" formatCode="#,##0.00&quot; €&quot;;[RED]\-#,##0.00&quot; €&quot;"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -163,6 +187,14 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -231,7 +263,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -309,6 +341,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1414,7 +1450,11 @@
       <c r="K20" s="17"/>
     </row>
     <row r="21" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C21" s="17"/>
+      <c r="A21" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
       <c r="D21" s="17"/>
       <c r="E21" s="17"/>
       <c r="F21" s="17"/>
@@ -1424,7 +1464,11 @@
       <c r="K21" s="17"/>
     </row>
     <row r="22" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C22" s="17"/>
+      <c r="A22" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
       <c r="D22" s="17"/>
       <c r="E22" s="17"/>
       <c r="F22" s="17"/>
@@ -1434,7 +1478,11 @@
       <c r="K22" s="17"/>
     </row>
     <row r="23" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C23" s="17"/>
+      <c r="A23" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
       <c r="D23" s="17"/>
       <c r="E23" s="17"/>
       <c r="F23" s="17"/>
@@ -1444,8 +1492,12 @@
       <c r="K23" s="17"/>
     </row>
     <row r="24" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
+      <c r="A24" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
       <c r="E24" s="17"/>
       <c r="F24" s="17"/>
       <c r="G24" s="17"/>
@@ -1454,7 +1506,11 @@
       <c r="K24" s="17"/>
     </row>
     <row r="25" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C25" s="17"/>
+      <c r="A25" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
       <c r="D25" s="17"/>
       <c r="E25" s="17"/>
       <c r="F25" s="17"/>
@@ -1464,7 +1520,11 @@
       <c r="K25" s="17"/>
     </row>
     <row r="26" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C26" s="17"/>
+      <c r="A26" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
       <c r="D26" s="17"/>
       <c r="E26" s="17"/>
       <c r="F26" s="17"/>
@@ -1474,7 +1534,11 @@
       <c r="K26" s="17"/>
     </row>
     <row r="27" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C27" s="17"/>
+      <c r="A27" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="19"/>
+      <c r="C27" s="19"/>
       <c r="D27" s="17"/>
       <c r="E27" s="17"/>
       <c r="F27" s="17"/>
@@ -1484,7 +1548,11 @@
       <c r="K27" s="17"/>
     </row>
     <row r="28" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C28" s="17"/>
+      <c r="A28" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
       <c r="D28" s="17"/>
       <c r="E28" s="17"/>
       <c r="F28" s="17"/>
@@ -11214,10 +11282,18 @@
       <c r="K1000" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="11">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="L15:M15"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Ajout du kpi_roi.xlsx et maj de l'estimation
</commit_message>
<xml_diff>
--- a/docs/cadrage/Estimation_NutriScope.xlsx
+++ b/docs/cadrage/Estimation_NutriScope.xlsx
@@ -263,7 +263,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -344,7 +344,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1377,6 +1381,10 @@
         <f aca="false">((K14/2)/1000000)*1.1</f>
         <v>275.914131904344</v>
       </c>
+      <c r="N14" s="0" t="n">
+        <f aca="false">SUM(N2:N13)</f>
+        <v>41805.1715006583</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C15" s="17"/>
@@ -1464,11 +1472,11 @@
       <c r="K21" s="17"/>
     </row>
     <row r="22" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
       <c r="D22" s="17"/>
       <c r="E22" s="17"/>
       <c r="F22" s="17"/>
@@ -1478,11 +1486,11 @@
       <c r="K22" s="17"/>
     </row>
     <row r="23" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="B23" s="19"/>
-      <c r="C23" s="19"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
       <c r="D23" s="17"/>
       <c r="E23" s="17"/>
       <c r="F23" s="17"/>
@@ -1492,12 +1500,12 @@
       <c r="K23" s="17"/>
     </row>
     <row r="24" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="19" t="s">
+      <c r="A24" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="19"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="21"/>
       <c r="E24" s="17"/>
       <c r="F24" s="17"/>
       <c r="G24" s="17"/>
@@ -1506,11 +1514,11 @@
       <c r="K24" s="17"/>
     </row>
     <row r="25" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="s">
+      <c r="A25" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21"/>
       <c r="D25" s="17"/>
       <c r="E25" s="17"/>
       <c r="F25" s="17"/>
@@ -1520,11 +1528,11 @@
       <c r="K25" s="17"/>
     </row>
     <row r="26" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="19" t="s">
+      <c r="A26" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
       <c r="D26" s="17"/>
       <c r="E26" s="17"/>
       <c r="F26" s="17"/>
@@ -1534,11 +1542,11 @@
       <c r="K26" s="17"/>
     </row>
     <row r="27" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="19" t="s">
+      <c r="A27" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B27" s="19"/>
-      <c r="C27" s="19"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
       <c r="D27" s="17"/>
       <c r="E27" s="17"/>
       <c r="F27" s="17"/>
@@ -1548,11 +1556,11 @@
       <c r="K27" s="17"/>
     </row>
     <row r="28" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="19" t="s">
+      <c r="A28" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
       <c r="D28" s="17"/>
       <c r="E28" s="17"/>
       <c r="F28" s="17"/>

</xml_diff>